<commit_message>
final version I used compiling the ma text
</commit_message>
<xml_diff>
--- a/ma_figures/comparison_table.xlsx
+++ b/ma_figures/comparison_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/matthew_gidden_pnnl_gov/Documents/Documents/work/papers/2024_gidden_cstorage/ma_figures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{E89A3F42-E1C6-6145-B0FC-E434B0424226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8EF2FF4-2BD0-9741-94EA-61C7191309E2}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{E89A3F42-E1C6-6145-B0FC-E434B0424226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C214F069-5486-4449-9E2D-322707834D61}"/>
   <bookViews>
     <workbookView xWindow="-10500" yWindow="-18900" windowWidth="27240" windowHeight="16440" xr2:uid="{A60DB7CB-DBC6-354C-BFB1-284D8AEDA6ED}"/>
   </bookViews>
@@ -78,8 +78,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -124,11 +125,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +518,7 @@
         <f>E2/C2</f>
         <v>0.71212121212121215</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="4">
         <f>E2/D2</f>
         <v>0.54230769230769227</v>
       </c>
@@ -542,7 +544,7 @@
         <f t="shared" ref="F3:F7" si="0">E3/C3</f>
         <v>0.41585365853658535</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="4">
         <f t="shared" ref="G3:G7" si="1">E3/D3</f>
         <v>0.12692307692307692</v>
       </c>
@@ -568,7 +570,7 @@
         <f t="shared" si="0"/>
         <v>9063.4920634920636</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="4">
         <f t="shared" si="1"/>
         <v>5.4380952380952383</v>
       </c>
@@ -594,7 +596,7 @@
         <f t="shared" si="0"/>
         <v>56507.936507936509</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="4">
         <f t="shared" si="1"/>
         <v>0.11558441558441558</v>
       </c>
@@ -620,7 +622,7 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="4">
         <f t="shared" si="1"/>
         <v>27.521367521367527</v>
       </c>
@@ -646,7 +648,7 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="4">
         <f t="shared" si="1"/>
         <v>0.39279588336192112</v>
       </c>

</xml_diff>